<commit_message>
Updating gitignore and Jegyezo
</commit_message>
<xml_diff>
--- a/Jegyező.xlsx
+++ b/Jegyező.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Egyetem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E286D10-8297-4100-B5EC-734798208605}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC22C37B-0920-4E32-B101-3C84D7A64BEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -384,19 +384,6 @@
         </r>
       </text>
     </comment>
-    <comment ref="AG2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000006000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Arial"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Csak 2. szemeszter</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="S3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000007000000}">
       <text>
         <r>
@@ -420,19 +407,6 @@
             <scheme val="minor"/>
           </rPr>
           <t>Csak 1. szemeszter</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AG3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000009000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Arial"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Csak 2. szemeszter</t>
         </r>
       </text>
     </comment>
@@ -503,32 +477,6 @@
         </r>
       </text>
     </comment>
-    <comment ref="AG8" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-00000E000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Arial"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Csak 2. szemeszter</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AG9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-00000F000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Arial"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Csak 2. szemeszter</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="A10" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000010000000}">
       <text>
         <r>
@@ -574,7 +522,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="211">
   <si>
     <t>2. félévben felvehető tárgyak</t>
   </si>
@@ -1188,10 +1136,25 @@
     <t>Mesterséges intelligencia</t>
   </si>
   <si>
-    <t>Összes</t>
-  </si>
-  <si>
     <t>Telekomunikációs hálózatok Gy</t>
+  </si>
+  <si>
+    <t>Numerikus módszerek II. Ea</t>
+  </si>
+  <si>
+    <t>Numerikus módszerek II. Gy</t>
+  </si>
+  <si>
+    <t>Valószínűségszámítás</t>
+  </si>
+  <si>
+    <t>Számítógépes grafika Gy</t>
+  </si>
+  <si>
+    <t>Térinformatika</t>
+  </si>
+  <si>
+    <t>Szakdolgozati konzultáció</t>
   </si>
 </sst>
 </file>
@@ -1584,7 +1547,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1702,14 +1665,16 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normál" xfId="0" builtinId="0"/>
@@ -1779,6 +1744,11 @@
       <tableStyleElement type="secondRowStripe" dxfId="4"/>
     </tableStyle>
   </tableStyles>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFE599"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -2988,10 +2958,10 @@
       </c>
     </row>
     <row r="2" spans="1:51" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A2" s="75" t="s">
+      <c r="A2" s="79" t="s">
         <v>45</v>
       </c>
-      <c r="B2" s="76"/>
+      <c r="B2" s="80"/>
       <c r="C2" s="3" t="s">
         <v>46</v>
       </c>
@@ -3138,8 +3108,8 @@
       </c>
     </row>
     <row r="3" spans="1:51" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A3" s="76"/>
-      <c r="B3" s="76"/>
+      <c r="A3" s="80"/>
+      <c r="B3" s="80"/>
       <c r="C3" s="3" t="s">
         <v>54</v>
       </c>
@@ -3286,8 +3256,8 @@
       </c>
     </row>
     <row r="4" spans="1:51" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A4" s="76"/>
-      <c r="B4" s="76"/>
+      <c r="A4" s="80"/>
+      <c r="B4" s="80"/>
       <c r="C4" s="3" t="s">
         <v>60</v>
       </c>
@@ -3434,8 +3404,8 @@
       </c>
     </row>
     <row r="5" spans="1:51" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A5" s="76"/>
-      <c r="B5" s="76"/>
+      <c r="A5" s="80"/>
+      <c r="B5" s="80"/>
       <c r="C5" s="3" t="s">
         <v>68</v>
       </c>
@@ -3582,8 +3552,8 @@
       </c>
     </row>
     <row r="6" spans="1:51" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A6" s="76"/>
-      <c r="B6" s="76"/>
+      <c r="A6" s="80"/>
+      <c r="B6" s="80"/>
       <c r="C6" s="3" t="s">
         <v>74</v>
       </c>
@@ -3728,8 +3698,8 @@
       </c>
     </row>
     <row r="7" spans="1:51" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A7" s="76"/>
-      <c r="B7" s="76"/>
+      <c r="A7" s="80"/>
+      <c r="B7" s="80"/>
       <c r="C7" s="3" t="s">
         <v>81</v>
       </c>
@@ -3874,8 +3844,8 @@
       </c>
     </row>
     <row r="8" spans="1:51" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A8" s="76"/>
-      <c r="B8" s="76"/>
+      <c r="A8" s="80"/>
+      <c r="B8" s="80"/>
       <c r="C8" s="3" t="s">
         <v>86</v>
       </c>
@@ -8905,7 +8875,7 @@
     <col min="49" max="49" width="4.44140625" customWidth="1" outlineLevel="1"/>
     <col min="50" max="50" width="4.44140625" bestFit="1" customWidth="1"/>
     <col min="51" max="51" width="4.21875" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="3.44140625" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:52" ht="13.2" x14ac:dyDescent="0.25">
@@ -9081,7 +9051,7 @@
         <v>29</v>
       </c>
       <c r="G2" s="60">
-        <f>AVERAGE(P2:P15)</f>
+        <f>AVERAGE(P:P)</f>
         <v>4.4285714285714288</v>
       </c>
       <c r="H2" s="6">
@@ -9189,37 +9159,41 @@
       <c r="AO2" s="9">
         <v>2</v>
       </c>
-      <c r="AP2" s="9"/>
+      <c r="AP2" s="9">
+        <v>2</v>
+      </c>
       <c r="AQ2" s="1">
         <f t="shared" ref="AQ2" si="12">IF(AP2 = 1,"",AO2)</f>
         <v>2</v>
       </c>
       <c r="AR2" s="1">
         <f t="shared" ref="AR2" si="13">IF(AP2 = 1,"",AP2)</f>
-        <v>0</v>
-      </c>
-      <c r="AS2" s="1" t="str">
+        <v>2</v>
+      </c>
+      <c r="AS2" s="1">
         <f t="shared" ref="AS2" si="14">IF(AO2*AP2=0,"",IF(AP2=1,"",AO2*AP2))</f>
-        <v/>
-      </c>
-      <c r="AU2" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="AV2" s="17">
-        <v>20</v>
-      </c>
-      <c r="AW2" s="17"/>
+        <v>4</v>
+      </c>
+      <c r="AU2" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="AV2" s="9">
+        <v>4</v>
+      </c>
+      <c r="AW2" s="9">
+        <v>3</v>
+      </c>
       <c r="AX2" s="1">
-        <f t="shared" ref="AX2:AX3" si="15">IF(AW2 = 1,"",AV2)</f>
-        <v>20</v>
+        <f>IF(AW2 = 1,"",AV2)</f>
+        <v>4</v>
       </c>
       <c r="AY2" s="1">
-        <f t="shared" ref="AY2:AY3" si="16">IF(AW2 = 1,"",AW2)</f>
-        <v>0</v>
-      </c>
-      <c r="AZ2" s="1" t="str">
-        <f t="shared" ref="AZ2:AZ23" si="17">IF(AV2*AW2=0,"",IF(AW2=1,"",AV2*AW2))</f>
-        <v/>
+        <f>IF(AW2 = 1,"",AW2)</f>
+        <v>3</v>
+      </c>
+      <c r="AZ2" s="1">
+        <f>IF(AV2*AW2=0,"",IF(AW2=1,"",AV2*AW2))</f>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:52" ht="13.2" x14ac:dyDescent="0.25">
@@ -9241,7 +9215,7 @@
         <v>33</v>
       </c>
       <c r="G3" s="63">
-        <f>AVERAGE(W2:W15)</f>
+        <f>AVERAGE(W:W)</f>
         <v>3.8</v>
       </c>
       <c r="H3" s="6">
@@ -9353,28 +9327,37 @@
         <v>5</v>
       </c>
       <c r="AQ3" s="1">
-        <f t="shared" ref="AQ3:AQ13" si="18">IF(AP3 = 1,"",AO3)</f>
+        <f t="shared" ref="AQ3:AQ13" si="15">IF(AP3 = 1,"",AO3)</f>
         <v>3</v>
       </c>
       <c r="AR3" s="1">
-        <f t="shared" ref="AR3:AR13" si="19">IF(AP3 = 1,"",AP3)</f>
+        <f t="shared" ref="AR3:AR13" si="16">IF(AP3 = 1,"",AP3)</f>
         <v>5</v>
       </c>
       <c r="AS3" s="1">
-        <f t="shared" ref="AS3:AS13" si="20">IF(AO3*AP3=0,"",IF(AP3=1,"",AO3*AP3))</f>
+        <f t="shared" ref="AS3:AS13" si="17">IF(AO3*AP3=0,"",IF(AP3=1,"",AO3*AP3))</f>
         <v>15</v>
       </c>
+      <c r="AU3" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="AV3" s="10">
+        <v>2</v>
+      </c>
+      <c r="AW3" s="10">
+        <v>2</v>
+      </c>
       <c r="AX3" s="1">
-        <f t="shared" si="15"/>
-        <v>0</v>
+        <f t="shared" ref="AX3:AX9" si="18">IF(AW3 = 1,"",AV3)</f>
+        <v>2</v>
       </c>
       <c r="AY3" s="1">
-        <f t="shared" si="16"/>
-        <v>0</v>
-      </c>
-      <c r="AZ3" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v/>
+        <f t="shared" ref="AY3:AY9" si="19">IF(AW3 = 1,"",AW3)</f>
+        <v>2</v>
+      </c>
+      <c r="AZ3" s="1">
+        <f t="shared" ref="AZ3:AZ9" si="20">IF(AV3*AW3=0,"",IF(AW3=1,"",AV3*AW3))</f>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:52" ht="13.2" x14ac:dyDescent="0.25">
@@ -9396,7 +9379,7 @@
         <v>25</v>
       </c>
       <c r="G4" s="63">
-        <f>AVERAGE(AD1:AD28)</f>
+        <f>AVERAGE(AD:AD)</f>
         <v>3.5555555555555554</v>
       </c>
       <c r="H4" s="6">
@@ -9504,24 +9487,41 @@
       <c r="AO4" s="10">
         <v>2</v>
       </c>
-      <c r="AP4" s="10"/>
-      <c r="AQ4" s="1">
+      <c r="AP4" s="10">
+        <v>1</v>
+      </c>
+      <c r="AQ4" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v/>
+      </c>
+      <c r="AR4" s="1" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+      <c r="AS4" s="1" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+      <c r="AU4" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="AV4" s="10">
+        <v>2</v>
+      </c>
+      <c r="AW4" s="10">
+        <v>3</v>
+      </c>
+      <c r="AX4" s="1">
         <f t="shared" si="18"/>
         <v>2</v>
       </c>
-      <c r="AR4" s="1">
+      <c r="AY4" s="1">
         <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-      <c r="AS4" s="1" t="str">
+        <v>3</v>
+      </c>
+      <c r="AZ4" s="1">
         <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="AX4" s="1"/>
-      <c r="AY4" s="1"/>
-      <c r="AZ4" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v/>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:52" ht="13.2" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>26</v>
       </c>
       <c r="G5" s="63">
-        <f>AVERAGE(AK1:AK39)</f>
+        <f>AVERAGE(AK:AK)</f>
         <v>4.0999999999999996</v>
       </c>
       <c r="H5" s="6">
@@ -9655,22 +9655,37 @@
         <v>4</v>
       </c>
       <c r="AQ5" s="1">
+        <f t="shared" si="15"/>
+        <v>4</v>
+      </c>
+      <c r="AR5" s="1">
+        <f t="shared" si="16"/>
+        <v>4</v>
+      </c>
+      <c r="AS5" s="1">
+        <f t="shared" si="17"/>
+        <v>16</v>
+      </c>
+      <c r="AU5" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="AV5" s="10">
+        <v>3</v>
+      </c>
+      <c r="AW5" s="10">
+        <v>4</v>
+      </c>
+      <c r="AX5" s="1">
         <f t="shared" si="18"/>
-        <v>4</v>
-      </c>
-      <c r="AR5" s="1">
+        <v>3</v>
+      </c>
+      <c r="AY5" s="1">
         <f t="shared" si="19"/>
         <v>4</v>
       </c>
-      <c r="AS5" s="1">
+      <c r="AZ5" s="1">
         <f t="shared" si="20"/>
-        <v>16</v>
-      </c>
-      <c r="AX5" s="1"/>
-      <c r="AY5" s="1"/>
-      <c r="AZ5" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v/>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:52" ht="13.2" x14ac:dyDescent="0.25">
@@ -9681,31 +9696,31 @@
       </c>
       <c r="D6" s="6">
         <f>IF(SUMPRODUCT(AR:AR,AQ:AQ)/SUM(AQ:AQ)=0,"",SUMPRODUCT(AR:AR,AQ:AQ)/SUM(AQ:AQ))</f>
-        <v>2.2777777777777777</v>
+        <v>3.3529411764705883</v>
       </c>
       <c r="E6" s="7">
         <f>SUM(AO:AO)</f>
-        <v>38.700000000000003</v>
+        <v>36</v>
       </c>
       <c r="F6" s="7">
         <f>SUMIFS(AO:AO,AP:AP,"&gt;1")</f>
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="G6" s="63">
-        <f>AVERAGE(AR2:AR38)</f>
-        <v>2</v>
+        <f>AVERAGE(AR:AR)</f>
+        <v>3.2727272727272729</v>
       </c>
       <c r="H6" s="6">
         <f>SUM(AS:AS)/30</f>
-        <v>2.7333333333333334</v>
+        <v>3.8</v>
       </c>
       <c r="I6" s="6">
         <f>SUM(AS:AS)/30*(F6/E6)</f>
-        <v>1.6950904392764858</v>
+        <v>3.5888888888888886</v>
       </c>
       <c r="J6" s="6">
         <f>SUM(Q:Q,X:X,AE:AE,AL:AL,AS:AS)/(30*5)*(SUM(F2:F6)/SUM(E2:E6))</f>
-        <v>3.1474154435226551</v>
+        <v>3.64</v>
       </c>
       <c r="K6" s="18" t="s">
         <v>167</v>
@@ -9800,24 +9815,41 @@
       <c r="AO6" s="10">
         <v>2</v>
       </c>
-      <c r="AP6" s="10"/>
+      <c r="AP6" s="10">
+        <v>2</v>
+      </c>
       <c r="AQ6" s="1">
+        <f t="shared" si="15"/>
+        <v>2</v>
+      </c>
+      <c r="AR6" s="1">
+        <f t="shared" si="16"/>
+        <v>2</v>
+      </c>
+      <c r="AS6" s="1">
+        <f t="shared" si="17"/>
+        <v>4</v>
+      </c>
+      <c r="AU6" s="75" t="s">
+        <v>208</v>
+      </c>
+      <c r="AV6" s="75">
+        <v>3</v>
+      </c>
+      <c r="AW6" s="75">
+        <v>5</v>
+      </c>
+      <c r="AX6" s="1">
         <f t="shared" si="18"/>
-        <v>2</v>
-      </c>
-      <c r="AR6" s="1">
+        <v>3</v>
+      </c>
+      <c r="AY6" s="1">
         <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-      <c r="AS6" s="1" t="str">
+        <v>5</v>
+      </c>
+      <c r="AZ6" s="1">
         <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="AX6" s="1"/>
-      <c r="AY6" s="1"/>
-      <c r="AZ6" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v/>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:52" ht="13.2" x14ac:dyDescent="0.25">
@@ -9826,33 +9858,33 @@
       <c r="C7" s="72" t="s">
         <v>81</v>
       </c>
-      <c r="D7" s="6" t="str">
+      <c r="D7" s="6">
         <f>IF(SUMPRODUCT(AY:AY,AX:AX)/SUM(AX:AX)=0,"",SUMPRODUCT(AY:AY,AX:AX)/SUM(AX:AX))</f>
-        <v/>
+        <v>4.4749999999999996</v>
       </c>
       <c r="E7" s="7">
         <f>SUM(AV:AV)</f>
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F7" s="7">
         <f>SUMIFS(AV:AV,AW:AW,"&gt;1")</f>
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="G7" s="63">
-        <f>AVERAGE(AY2:AY30)</f>
-        <v>0</v>
+        <f>AVERAGE(AY:AY)</f>
+        <v>4</v>
       </c>
       <c r="H7" s="6">
         <f>SUM(AZ:AZ)/30</f>
-        <v>0</v>
+        <v>5.9666666666666668</v>
       </c>
       <c r="I7" s="6">
         <f>SUM(AZ:AZ)/30*(F7/E7)</f>
-        <v>0</v>
+        <v>5.9666666666666668</v>
       </c>
       <c r="J7" s="6">
         <f>SUM(Q:Q,X:X,AE:AE,AL:AL,AS:AS,AZ:AZ)/(30*6)*(SUM(F2:F7)/SUM(E2:E7))</f>
-        <v>2.3259762308998306</v>
+        <v>4.0216781214203898</v>
       </c>
       <c r="K7" s="20" t="s">
         <v>187</v>
@@ -9899,13 +9931,13 @@
         <f t="shared" si="5"/>
         <v>10</v>
       </c>
-      <c r="Z7" s="19" t="s">
+      <c r="Z7" s="15" t="s">
         <v>175</v>
       </c>
-      <c r="AA7" s="19">
+      <c r="AA7" s="15">
         <v>2</v>
       </c>
-      <c r="AB7" s="19">
+      <c r="AB7" s="15">
         <v>3</v>
       </c>
       <c r="AC7" s="1">
@@ -9951,22 +9983,37 @@
         <v>3</v>
       </c>
       <c r="AQ7" s="1">
+        <f t="shared" si="15"/>
+        <v>3</v>
+      </c>
+      <c r="AR7" s="1">
+        <f t="shared" si="16"/>
+        <v>3</v>
+      </c>
+      <c r="AS7" s="1">
+        <f t="shared" si="17"/>
+        <v>9</v>
+      </c>
+      <c r="AU7" s="75" t="s">
+        <v>209</v>
+      </c>
+      <c r="AV7" s="75">
+        <v>4</v>
+      </c>
+      <c r="AW7" s="75">
+        <v>5</v>
+      </c>
+      <c r="AX7" s="1">
         <f t="shared" si="18"/>
-        <v>3</v>
-      </c>
-      <c r="AR7" s="1">
+        <v>4</v>
+      </c>
+      <c r="AY7" s="1">
         <f t="shared" si="19"/>
-        <v>3</v>
-      </c>
-      <c r="AS7" s="1">
+        <v>5</v>
+      </c>
+      <c r="AZ7" s="1">
         <f t="shared" si="20"/>
-        <v>9</v>
-      </c>
-      <c r="AX7" s="1"/>
-      <c r="AY7" s="1"/>
-      <c r="AZ7" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v/>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:52" ht="13.2" x14ac:dyDescent="0.25">
@@ -9977,28 +10024,31 @@
       </c>
       <c r="D8" s="21">
         <f>SUMPRODUCT(D2:D7,E2:E7)/SUMIF(D2:D7,"&gt; 0",E2:E7)</f>
-        <v>3.6001914486279518</v>
+        <v>3.998483929654336</v>
       </c>
       <c r="E8" s="22">
         <f t="shared" ref="E8:F8" si="21">SUM(E2:E7)</f>
-        <v>176.7</v>
+        <v>194</v>
       </c>
       <c r="F8" s="22">
         <f t="shared" si="21"/>
-        <v>137</v>
+        <v>187</v>
       </c>
       <c r="G8" s="66">
-        <f>AVERAGE(P2:P25,W2:W25,AD2:AD29)</f>
-        <v>3.8846153846153846</v>
-      </c>
-      <c r="H8" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="I8" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="J8" s="22" t="s">
-        <v>20</v>
+        <f>AVERAGE(G2:G7)</f>
+        <v>3.8594757094757095</v>
+      </c>
+      <c r="H8" s="66">
+        <f>AVERAGE(H2:H7)</f>
+        <v>4.1722222222222216</v>
+      </c>
+      <c r="I8" s="66">
+        <f t="shared" ref="I8:J8" si="22">AVERAGE(I2:I7)</f>
+        <v>4.0537037037037038</v>
+      </c>
+      <c r="J8" s="66">
+        <f t="shared" si="22"/>
+        <v>3.924328241722034</v>
       </c>
       <c r="K8" s="61" t="s">
         <v>47</v>
@@ -10045,13 +10095,13 @@
         <f t="shared" si="5"/>
         <v>12</v>
       </c>
-      <c r="Z8" s="19" t="s">
+      <c r="Z8" s="15" t="s">
         <v>180</v>
       </c>
-      <c r="AA8" s="19">
+      <c r="AA8" s="15">
         <v>3</v>
       </c>
-      <c r="AB8" s="19">
+      <c r="AB8" s="15">
         <v>4</v>
       </c>
       <c r="AC8" s="1">
@@ -10097,22 +10147,37 @@
         <v>2</v>
       </c>
       <c r="AQ8" s="1">
+        <f t="shared" si="15"/>
+        <v>4</v>
+      </c>
+      <c r="AR8" s="1">
+        <f t="shared" si="16"/>
+        <v>2</v>
+      </c>
+      <c r="AS8" s="1">
+        <f t="shared" si="17"/>
+        <v>8</v>
+      </c>
+      <c r="AU8" s="76" t="s">
+        <v>192</v>
+      </c>
+      <c r="AV8" s="76">
+        <v>2</v>
+      </c>
+      <c r="AW8" s="76">
+        <v>5</v>
+      </c>
+      <c r="AX8" s="1">
         <f t="shared" si="18"/>
-        <v>4</v>
-      </c>
-      <c r="AR8" s="1">
+        <v>2</v>
+      </c>
+      <c r="AY8" s="1">
         <f t="shared" si="19"/>
-        <v>2</v>
-      </c>
-      <c r="AS8" s="1">
+        <v>5</v>
+      </c>
+      <c r="AZ8" s="1">
         <f t="shared" si="20"/>
-        <v>8</v>
-      </c>
-      <c r="AX8" s="1"/>
-      <c r="AY8" s="1"/>
-      <c r="AZ8" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v/>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:52" ht="13.2" x14ac:dyDescent="0.25">
@@ -10183,53 +10248,68 @@
         <f t="shared" si="8"/>
         <v>15</v>
       </c>
-      <c r="AG9" s="10" t="s">
-        <v>192</v>
-      </c>
-      <c r="AH9" s="10">
-        <v>2</v>
-      </c>
-      <c r="AI9" s="10">
-        <v>5</v>
+      <c r="AG9" s="19" t="s">
+        <v>193</v>
+      </c>
+      <c r="AH9" s="19">
+        <v>3</v>
+      </c>
+      <c r="AI9" s="19">
+        <v>4</v>
       </c>
       <c r="AJ9" s="1">
         <f t="shared" si="9"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AK9" s="1">
         <f t="shared" si="10"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AL9" s="1">
         <f t="shared" si="11"/>
-        <v>10</v>
-      </c>
-      <c r="AN9" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="AN9" s="15" t="s">
         <v>202</v>
       </c>
-      <c r="AO9" s="10">
+      <c r="AO9" s="15">
         <v>2</v>
       </c>
-      <c r="AP9" s="10">
+      <c r="AP9" s="15">
         <v>2</v>
       </c>
       <c r="AQ9" s="1">
+        <f t="shared" si="15"/>
+        <v>2</v>
+      </c>
+      <c r="AR9" s="1">
+        <f t="shared" si="16"/>
+        <v>2</v>
+      </c>
+      <c r="AS9" s="1">
+        <f t="shared" si="17"/>
+        <v>4</v>
+      </c>
+      <c r="AU9" s="76" t="s">
+        <v>210</v>
+      </c>
+      <c r="AV9" s="76">
+        <v>20</v>
+      </c>
+      <c r="AW9" s="76">
+        <v>5</v>
+      </c>
+      <c r="AX9" s="1">
         <f t="shared" si="18"/>
-        <v>2</v>
-      </c>
-      <c r="AR9" s="1">
+        <v>20</v>
+      </c>
+      <c r="AY9" s="1">
         <f t="shared" si="19"/>
-        <v>2</v>
-      </c>
-      <c r="AS9" s="1">
+        <v>5</v>
+      </c>
+      <c r="AZ9" s="1">
         <f t="shared" si="20"/>
-        <v>4</v>
-      </c>
-      <c r="AX9" s="1"/>
-      <c r="AY9" s="1"/>
-      <c r="AZ9" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v/>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:52" ht="13.2" x14ac:dyDescent="0.25">
@@ -10287,13 +10367,13 @@
         <v>6</v>
       </c>
       <c r="AG10" s="19" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AH10" s="19">
         <v>3</v>
       </c>
       <c r="AI10" s="19">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AJ10" s="1">
         <f t="shared" si="9"/>
@@ -10301,39 +10381,36 @@
       </c>
       <c r="AK10" s="1">
         <f t="shared" si="10"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AL10" s="1">
         <f t="shared" si="11"/>
-        <v>12</v>
-      </c>
-      <c r="AN10" s="10" t="s">
-        <v>205</v>
-      </c>
-      <c r="AO10" s="10">
+        <v>15</v>
+      </c>
+      <c r="AN10" s="15" t="s">
+        <v>204</v>
+      </c>
+      <c r="AO10" s="15">
         <v>3</v>
       </c>
-      <c r="AP10" s="10">
+      <c r="AP10" s="15">
         <v>5</v>
       </c>
       <c r="AQ10" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="15"/>
         <v>3</v>
       </c>
       <c r="AR10" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="16"/>
         <v>5</v>
       </c>
       <c r="AS10" s="1">
-        <f t="shared" si="20"/>
+        <f t="shared" si="17"/>
         <v>15</v>
       </c>
       <c r="AX10" s="1"/>
       <c r="AY10" s="1"/>
-      <c r="AZ10" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
+      <c r="AZ10" s="1"/>
     </row>
     <row r="11" spans="1:52" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
@@ -10388,18 +10465,18 @@
         <f t="shared" si="8"/>
         <v>8</v>
       </c>
-      <c r="AG11" s="19" t="s">
-        <v>194</v>
-      </c>
-      <c r="AH11" s="19">
-        <v>3</v>
-      </c>
-      <c r="AI11" s="19">
+      <c r="AG11" s="76" t="s">
+        <v>192</v>
+      </c>
+      <c r="AH11" s="76">
+        <v>2</v>
+      </c>
+      <c r="AI11" s="76">
         <v>5</v>
       </c>
       <c r="AJ11" s="1">
         <f t="shared" si="9"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AK11" s="1">
         <f t="shared" si="10"/>
@@ -10407,33 +10484,32 @@
       </c>
       <c r="AL11" s="1">
         <f t="shared" si="11"/>
-        <v>15</v>
-      </c>
-      <c r="AN11" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="AN11" s="15" t="s">
         <v>201</v>
       </c>
-      <c r="AO11" s="10">
+      <c r="AO11" s="15">
         <v>3</v>
       </c>
-      <c r="AP11" s="10"/>
+      <c r="AP11" s="15">
+        <v>3</v>
+      </c>
       <c r="AQ11" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="15"/>
         <v>3</v>
       </c>
       <c r="AR11" s="1">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-      <c r="AS11" s="1" t="str">
-        <f t="shared" si="20"/>
-        <v/>
+        <f t="shared" si="16"/>
+        <v>3</v>
+      </c>
+      <c r="AS11" s="1">
+        <f t="shared" si="17"/>
+        <v>9</v>
       </c>
       <c r="AX11" s="1"/>
       <c r="AY11" s="1"/>
-      <c r="AZ11" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
+      <c r="AZ11" s="1"/>
     </row>
     <row r="12" spans="1:52" ht="13.2" x14ac:dyDescent="0.25">
       <c r="E12" s="1"/>
@@ -10478,33 +10554,30 @@
       <c r="AJ12" s="1"/>
       <c r="AK12" s="1"/>
       <c r="AL12" s="1"/>
-      <c r="AN12" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="AO12" s="10">
+      <c r="AN12" s="19" t="s">
+        <v>203</v>
+      </c>
+      <c r="AO12" s="19">
+        <v>3</v>
+      </c>
+      <c r="AP12" s="19">
         <v>5</v>
       </c>
-      <c r="AP12" s="10">
+      <c r="AQ12" s="1">
+        <f t="shared" si="15"/>
         <v>3</v>
       </c>
-      <c r="AQ12" s="1">
-        <f t="shared" si="18"/>
+      <c r="AR12" s="1">
+        <f t="shared" si="16"/>
         <v>5</v>
       </c>
-      <c r="AR12" s="1">
-        <f t="shared" si="19"/>
-        <v>3</v>
-      </c>
       <c r="AS12" s="1">
-        <f t="shared" si="20"/>
+        <f t="shared" si="17"/>
         <v>15</v>
       </c>
       <c r="AX12" s="1"/>
       <c r="AY12" s="1"/>
-      <c r="AZ12" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
+      <c r="AZ12" s="1"/>
     </row>
     <row r="13" spans="1:52" ht="13.2" x14ac:dyDescent="0.25">
       <c r="E13" s="1"/>
@@ -10526,31 +10599,30 @@
       <c r="AJ13" s="1"/>
       <c r="AK13" s="1"/>
       <c r="AL13" s="1"/>
-      <c r="AN13" s="10" t="s">
-        <v>203</v>
-      </c>
-      <c r="AO13" s="10">
+      <c r="AN13" s="75" t="s">
+        <v>15</v>
+      </c>
+      <c r="AO13" s="75">
+        <v>5</v>
+      </c>
+      <c r="AP13" s="75">
         <v>3</v>
       </c>
-      <c r="AP13" s="10"/>
       <c r="AQ13" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="15"/>
+        <v>5</v>
+      </c>
+      <c r="AR13" s="1">
+        <f t="shared" si="16"/>
         <v>3</v>
       </c>
-      <c r="AR13" s="1">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-      <c r="AS13" s="1" t="str">
-        <f t="shared" si="20"/>
-        <v/>
+      <c r="AS13" s="1">
+        <f t="shared" si="17"/>
+        <v>15</v>
       </c>
       <c r="AX13" s="1"/>
       <c r="AY13" s="1"/>
-      <c r="AZ13" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
+      <c r="AZ13" s="1"/>
     </row>
     <row r="14" spans="1:52" ht="13.2" x14ac:dyDescent="0.25">
       <c r="E14" s="1"/>
@@ -10577,10 +10649,7 @@
       <c r="AS14" s="1"/>
       <c r="AX14" s="1"/>
       <c r="AY14" s="1"/>
-      <c r="AZ14" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
+      <c r="AZ14" s="1"/>
     </row>
     <row r="15" spans="1:52" ht="13.2" x14ac:dyDescent="0.25">
       <c r="E15" s="1"/>
@@ -10600,6 +10669,7 @@
       <c r="AB15" s="1"/>
       <c r="AC15" s="1"/>
       <c r="AE15" s="1"/>
+      <c r="AG15" s="1"/>
       <c r="AJ15" s="1"/>
       <c r="AK15" s="1"/>
       <c r="AL15" s="1"/>
@@ -10609,7 +10679,7 @@
       <c r="AX15" s="1"/>
       <c r="AY15" s="1"/>
       <c r="AZ15" s="1" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" ref="AZ15:AZ23" si="23">IF(AV15*AW15=0,"",IF(AW15=1,"",AV15*AW15))</f>
         <v/>
       </c>
     </row>
@@ -10640,7 +10710,7 @@
       <c r="AX16" s="1"/>
       <c r="AY16" s="1"/>
       <c r="AZ16" s="1" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
     </row>
@@ -10662,26 +10732,15 @@
       <c r="AH17" s="1"/>
       <c r="AI17" s="1"/>
       <c r="AJ17" s="1"/>
-      <c r="AK17" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="AM17">
-        <v>45</v>
-      </c>
-      <c r="AN17" s="1">
-        <f>$AM$17 * AO17 - $AM$18</f>
-        <v>18.25</v>
-      </c>
-      <c r="AO17">
-        <v>0.85</v>
-      </c>
+      <c r="AK17" s="1"/>
+      <c r="AN17" s="1"/>
       <c r="AQ17" s="1"/>
       <c r="AR17" s="1"/>
       <c r="AS17" s="1"/>
       <c r="AX17" s="1"/>
       <c r="AY17" s="1"/>
       <c r="AZ17" s="1" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
     </row>
@@ -10696,27 +10755,16 @@
       <c r="AD18" s="1"/>
       <c r="AE18" s="1"/>
       <c r="AJ18" s="1"/>
-      <c r="AK18" s="1" t="s">
-        <v>167</v>
-      </c>
+      <c r="AK18" s="1"/>
       <c r="AL18" s="1"/>
-      <c r="AM18">
-        <v>20</v>
-      </c>
-      <c r="AN18" s="1">
-        <f t="shared" ref="AN18:AN20" si="22">$AM$17 * AO18 - $AM$18</f>
-        <v>13.75</v>
-      </c>
-      <c r="AO18">
-        <v>0.75</v>
-      </c>
+      <c r="AN18" s="1"/>
       <c r="AQ18" s="1"/>
       <c r="AR18" s="1"/>
       <c r="AS18" s="1"/>
       <c r="AX18" s="1"/>
       <c r="AY18" s="1"/>
       <c r="AZ18" s="1" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
     </row>
@@ -10732,24 +10780,15 @@
       <c r="AE19" s="1"/>
       <c r="AJ19" s="1"/>
       <c r="AK19" s="1"/>
-      <c r="AL19" s="1" t="str">
-        <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="AN19" s="1">
-        <f t="shared" si="22"/>
-        <v>7</v>
-      </c>
-      <c r="AO19">
-        <v>0.6</v>
-      </c>
+      <c r="AL19" s="1"/>
+      <c r="AN19" s="1"/>
       <c r="AQ19" s="1"/>
       <c r="AR19" s="1"/>
       <c r="AS19" s="1"/>
       <c r="AX19" s="1"/>
       <c r="AY19" s="1"/>
       <c r="AZ19" s="1" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
     </row>
@@ -10768,24 +10807,15 @@
       <c r="AE20" s="1"/>
       <c r="AJ20" s="1"/>
       <c r="AK20" s="1"/>
-      <c r="AL20" s="1" t="str">
-        <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="AN20" s="1">
-        <f t="shared" si="22"/>
-        <v>2.5</v>
-      </c>
-      <c r="AO20">
-        <v>0.5</v>
-      </c>
+      <c r="AL20" s="1"/>
+      <c r="AN20" s="1"/>
       <c r="AQ20" s="1"/>
       <c r="AR20" s="1"/>
       <c r="AS20" s="1"/>
       <c r="AX20" s="1"/>
       <c r="AY20" s="1"/>
       <c r="AZ20" s="1" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
     </row>
@@ -10812,7 +10842,7 @@
       <c r="AX21" s="1"/>
       <c r="AY21" s="1"/>
       <c r="AZ21" s="1" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
     </row>
@@ -10842,7 +10872,7 @@
       <c r="AX22" s="1"/>
       <c r="AY22" s="1"/>
       <c r="AZ22" s="1" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
     </row>
@@ -10871,7 +10901,7 @@
       <c r="AX23" s="1"/>
       <c r="AY23" s="1"/>
       <c r="AZ23" s="1" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
     </row>
@@ -10949,7 +10979,7 @@
       <c r="V27" s="1"/>
       <c r="W27" s="1"/>
       <c r="X27" s="70" t="str">
-        <f t="shared" ref="X27:X32" si="23">IF(T27*U27=0,"",T27*U27)</f>
+        <f t="shared" ref="X27:X32" si="24">IF(T27*U27=0,"",T27*U27)</f>
         <v/>
       </c>
       <c r="Y27" s="70"/>
@@ -10999,7 +11029,7 @@
       <c r="V28" s="1"/>
       <c r="W28" s="1"/>
       <c r="X28" s="70" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="Y28" s="70"/>
@@ -11036,7 +11066,7 @@
       <c r="V29" s="1"/>
       <c r="W29" s="1"/>
       <c r="X29" s="70" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="Y29" s="70"/>
@@ -11070,7 +11100,7 @@
       <c r="V30" s="1"/>
       <c r="W30" s="1"/>
       <c r="X30" s="70" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="Y30" s="70"/>
@@ -11107,7 +11137,7 @@
       <c r="V31" s="1"/>
       <c r="W31" s="1"/>
       <c r="X31" s="70" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="Y31" s="70"/>
@@ -11144,7 +11174,7 @@
       <c r="V32" s="1"/>
       <c r="W32" s="1"/>
       <c r="X32" s="70" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
       <c r="Y32" s="70"/>
@@ -15166,7 +15196,7 @@
       <formula>2.75</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations disablePrompts="1" count="2">
     <dataValidation type="decimal" allowBlank="1" showDropDown="1" showErrorMessage="1" sqref="N2:N10 N25:N1000" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>1</formula1>
       <formula2>5</formula2>

</xml_diff>